<commit_message>
Phase 2: seed Search Log with batch-1 search audit trail
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EDRVMJpCj9m8Xg2jAMcbUq
</commit_message>
<xml_diff>
--- a/output/Gregory_Reinhart_Job_Search_Tracker.xlsx
+++ b/output/Gregory_Reinhart_Job_Search_Tracker.xlsx
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -955,7 +955,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -968,7 +967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1143,7 +1142,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:AB1"/>
   <conditionalFormatting sqref="P2:P500">
@@ -1194,7 +1192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1261,7 +1259,266 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Marketing Operations Specialist</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0-30d (default)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Indeed default recency broad; many stale/junior</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Marketing Operations Analyst</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0-30d</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Mostly BA/Data Analyst noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Campaign Operations Specialist</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Campaign Operations</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0-30d</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>CRM/RevOps + agency noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Marketing Operations Specialist (REMOTE, FT)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0-8d</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>5 of 886</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Salaries skew low $50-76k; verify seniority</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Marketing Operations (Remote, 7d)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0-7d</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>20 of 142</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Dice engineering-heavy; low signal for MarOps — deprioritized</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1274,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1365,7 +1622,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <dataValidations count="1">
@@ -1383,7 +1639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1474,7 +1730,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <dataValidations count="2">
@@ -1495,7 +1750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1556,7 +1811,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1569,7 +1823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1624,7 +1878,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1668,14 +1921,12 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Why are you interested in this role?</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Motivation</t>
@@ -1693,7 +1944,6 @@
           <t>Why this company?</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Motivation</t>
@@ -1711,7 +1961,6 @@
           <t>Describe relevant experience.</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Experience</t>
@@ -1729,7 +1978,6 @@
           <t>Describe a process improvement.</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Experience</t>
@@ -1747,7 +1995,6 @@
           <t>Describe experience with CRM or marketing systems.</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Systems</t>
@@ -1765,7 +2012,6 @@
           <t>Describe experience with data accuracy or QA.</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Systems</t>
@@ -1783,7 +2029,6 @@
           <t>Describe experience working cross-functionally.</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Experience</t>
@@ -1801,7 +2046,6 @@
           <t>Describe experience with AI or automation.</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>AI</t>
@@ -1885,7 +2129,6 @@
           <t>Remote-work experience</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Logistics</t>
@@ -1975,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2036,7 +2279,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Phase 2-4: populate Job Pipeline with 31 verified-unique candidates
- 5-cluster parallel search (Indeed/ZipRecruiter/Dice/web) across all Tier 1-3 role families
- Deduplicated to 31 canonical records; provisional fit scores, tiers, recommendations
- 5 PRIORITY APPLY (Paylocity, Allstate, SureCost, Progressive, 1Password)
- Dashboard metrics updated (avg fit 72.4)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EDRVMJpCj9m8Xg2jAMcbUq
</commit_message>
<xml_diff>
--- a/output/Gregory_Reinhart_Job_Search_Tracker.xlsx
+++ b/output/Gregory_Reinhart_Job_Search_Tracker.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,10 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -103,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +123,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -578,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -612,7 +617,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -646,7 +651,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -882,7 +887,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0</v>
+        <v>72.40000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -967,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1139,6 +1144,3788 @@
       <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>Duplicate Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GR-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Marketing Operations Manager, Campaigns</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Paylocity</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>$83,000-$108,000</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Paylocity careers</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>https://www.paylocity.com/company/careers/all-listings.job.38338/</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>https://www.paylocity.com/company/careers/all-listings.job.38338/</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Marketing/Campaign Operations</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>PRIORITY APPLY</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Campaign lifecycle QA/pacing/reconciliation; Salesforce+HubSpot data integrity; UTM/attribution</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Deep HubSpot build depth; net-new 6sense/SalesLoft</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Standard B2B cadence</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>paylocity|marketing operations manager, campaigns</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GR-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Associate Manager, Operations, Governance &amp; AI Enablement</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Allstate</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>$75,100-$126,325</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Allstate Workday</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>https://allstate.wd5.myworkdayjobs.com/allstate_careers/job/us---remote/associate-manager--operations--governance---ai-enablement_r32227</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>https://allstate.wd5.myworkdayjobs.com/allstate_careers/job/us---remote/associate-manager--operations--governance---ai-enablement_r32227</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>AI Operations/Governance</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>84</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>PRIORITY APPLY</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>AI-assisted SOP/documentation + governance; process improvement; Power BI + finance QA</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Confirm IC not people-mgmt; grants software domain</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Scope creep toward supervision</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>allstate|associate manager, operations, governance &amp; ai enablement</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GR-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Marketing Operations Manager</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SureCost</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Remote US (select states)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes (OH listed)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>$100,000-$105,000</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ZipRecruiter/employer</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.surecost.com/careers</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.surecost.com/careers</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>83</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>PRIORITY APPLY</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Omnichannel campaign QA/reporting; healthcare-adjacent (pharmacy SaaS); Power BI/Tableau + data integrity</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>May want MAP platform ownership (Marketo/HubSpot admin)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Small team broad ownership</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>surecost|marketing operations manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GR-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Marketing Process Analyst Senior</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Progressive</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Ohio (remote; HQ Mayfield Village)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Remote US; occasional HQ travel</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Yes (Akron in radius)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>$81,400-$108,500</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Progressive careers</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>https://careers.progressive.com/en/jobs/17252889-marketing-process-analyst-senior/</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>https://careers.progressive.com/en/jobs/17252889-marketing-process-analyst-senior/</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Business Process Improvement</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P5" t="n">
+        <v>83</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>PRIORITY APPLY</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Marketing/CRM process analysis; XLOOKUP automation (4hr-&gt;15min); GA4/GTM + Power BI/Tableau</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>No formal Agile/Jira cert; partners with IT on experiments</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Occasional HQ travel; Agile-adjacent</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>progressive|marketing process analyst senior</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GR-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Senior Revenue Operations Analyst, Campaign Operations</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1Password</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Remote-first US</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>$92,000-$124,000</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1Password Ashby</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.accel.com/companies/1password/jobs/63901867-senior-revenue-operations-analyst-campaign-operations</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.accel.com/companies/1password/jobs/63901867-senior-revenue-operations-analyst-campaign-operations</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Campaign Operations</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>82</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>PRIORITY APPLY</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Campaign trafficking/QA/reconciliation/reporting; Salesforce hands-on; SOP/campaign governance</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>'Senior' attribution/routing depth; SQL training only</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Minor periodic travel</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>1password|senior revenue operations analyst, campaign operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GR-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Marketing Operations &amp; Project Manager</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Propelus</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Remote US (HQ Boulder CO)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Likely (verify)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>$80,000-$100,000</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Propelus Ashby</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/propelus/5b896559-34ee-4159-b295-e793e44c394a</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/propelus/5b896559-34ee-4159-b295-e793e44c394a</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Monday.com + HubSpot exact tools; SOP/process backbone; healthcare-compliance domain</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>PM tooling/cadence ownership; mentoring (confirm IC)</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Do-everything scope drift</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>propelus|marketing operations &amp; project manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GR-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sales Operations Analyst 3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Vermont Information Processing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Remote US (Colchester VT)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Full-time direct-hire</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>$81,600-$96,000</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aavqd9pj492p</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aavqd9pj492p</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Revenue Operations</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>HubSpot data integrity; pipeline/forecast dashboards; HubSpot RevOps cert</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Supports quota sales team (pref); light quote creation</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Drug screen/background check</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>vermont information processing|sales operations analyst 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GR-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Marketing Operations Analyst</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Avetta, LLC</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Likely (verify)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>$83,000-$109,000</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ZipRecruiter/Built In</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.avetta.com/careers</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.avetta.com/careers</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>KPI packages/marketing performance reporting; process improvement + data integrity; month-end reconciliation</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>May want Marketo/SF Marketing Cloud depth; SaaS-native pref</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Verify listing currently open</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>avetta, llc|marketing operations analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GR-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Data Analyst, Pharma/Health &amp; Wellness Media</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>M3 USA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Remote US (HQ Fort Washington PA)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>M3 SmartRecruiters</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/M3USA/744000063104061-data-analyst-pharma-health-and-wellness-media-remote-</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/M3USA/744000063104061-data-analyst-pharma-health-and-wellness-media-remote-</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Marketing Analytics/Media</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>77</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Healthcare media campaign analytics; Tableau + Power BI + GA4; pacing/segmentation reporting</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>DS/Stats degree pref; A/B testing; production SQL gap</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>In-house, low risk</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>m3 usa|data analyst, pharma/health &amp; wellness media</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GR-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Marketing Operations Manager</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Viz.ai</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Likely (verify)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>$107,100-$140,000</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ZipRecruiter/employer</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.viz.ai/jobs</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.viz.ai/jobs</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Marketing Operations</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>77</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Healthcare-AI; Salesforce data integrity; KPI reporting Power BI/Tableau</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Pardot (not claimable); confirm IC vs Senior/people-mgmt</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Verify posting live (cached closed)</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>viz.ai|marketing operations manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GR-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Revenue Operations Analyst (CRM &amp; Data Systems)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>AccuWeather</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Remote US (State College PA)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Remote available US</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/accuweather/jobs/7914946</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/accuweather/jobs/7914946</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Revenue Operations/CRM Ops</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>2</v>
+      </c>
+      <c r="P12" t="n">
+        <v>76</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Data integrity across revenue systems; HubSpot admin; attribution dashboards; no CPQ/Flow</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Dynamics 'as needed'; Clay enrichment new</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Older posting; confirm open + comp</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>accuweather|revenue operations analyst (crm &amp; data systems)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GR-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Revenue Operations Analyst</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Campaign Monitor (Marigold)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>$70,000-$80,000</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Marigold Workday</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>https://campaignmonitor.wd5.myworkdayjobs.com/marigold/job/remote-united-states/revenue-operations-analyst_r2443</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>https://campaignmonitor.wd5.myworkdayjobs.com/marigold/job/remote-united-states/revenue-operations-analyst_r2443</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Revenue Operations</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Marketing ops + Salesforce + reporting; martech-vendor narrative bridge; HubSpot RevOps cert</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Verify CPQ scope; comp below MBA band</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Entry/associate framing</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>campaign monitor (marigold)|revenue operations analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GR-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Marketing Performance Analyst</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Arctic Wolf</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>~$105,500-$108,500</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Arctic Wolf Workday</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>https://arcticwolf.wd1.myworkdayjobs.com/External</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>https://arcticwolf.wd1.myworkdayjobs.com/External</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Marketing BI/Analytics</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Power BI/Tableau funnel dashboards; ROI/finance partnering; HubSpot RevOps cert</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>B2B SaaS pipeline/attribution newer; some SQL</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Recency ambiguous - verify live</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>arctic wolf|marketing performance analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GR-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GTM Operations Manager</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>On The Stage</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Remote US (NY)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>SmartRecruiters</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/OnTheStage/744000136114322-gtm-operations-manager-remote</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/OnTheStage/744000136114322-gtm-operations-manager-remote</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>GTM Operations</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>2</v>
+      </c>
+      <c r="P15" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Audit/document/improve GTM workflows; SF/HubSpot data quality; dashboards</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Hands-on SF admin config; smaller company</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Confirm not build-the-function-solo</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>on the stage|gtm operations manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GR-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Revenue Operations Analyst</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>KPA</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Remote US (HQ Lafayette CO)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>From $75,000</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ZipRecruiter/employer</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.kpa.io/company/careers</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.kpa.io/company/careers</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Revenue Operations</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>2</v>
+      </c>
+      <c r="P16" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>HubSpot RevOps cert; Salesforce/Advendio integrity; XLOOKUP + reporting; compliance-software domain</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Some RevOps want production SQL/admin config</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Confirm ops not sales-enablement/quota</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>kpa|revenue operations analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GR-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Marketing Specialist (HubSpot Specialization)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Decisely</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Remote US (Alpharetta GA)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>100% remote</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>$85,000-$100,000</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.decisely.com</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.decisely.com</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Marketing Automation (HubSpot)</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P17" t="n">
+        <v>72</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>APPLY WITH TAILORING</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>HubSpot automation/workflows + RevOps cert; multi-channel campaign execution</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Heavy copywriting/creative + paid-media buying</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Generalist load dilutes ops focus</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>decisely|marketing specialist (hubspot specialization)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GR-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GTM Operations Analyst (Marketing)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CreatorIQ</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Remote US (verify US)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>~$71K-$116K market</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>CreatorIQ Ashby</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/creatoriq/43495f0e-71d1-4077-a5ed-76c3ccb92c6f</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/creatoriq/43495f0e-71d1-4077-a5ed-76c3ccb92c6f</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Demand Gen Operations</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>2</v>
+      </c>
+      <c r="P18" t="n">
+        <v>72</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Salesforce + HubSpot RevOps cert; data hygiene/reporting; lead-flow coordination</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>3+ yrs SaaS MarOps + deep HubSpot admin; Clay</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Confirm US-remote eligibility</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>creatoriq|gtm operations analyst (marketing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GR-018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Senior Business Process Analyst</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Pacific Life Insurance</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Remote US (HQ Omaha NE)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Remote optional US</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>$97,500-$134,000</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pacificlife.com/about-us/careers.html</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pacificlife.com/about-us/careers.html</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Business Process Improvement</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>2</v>
+      </c>
+      <c r="P19" t="n">
+        <v>72</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>SOP/process docs + audited reporting; budget/financial controls; XLOOKUP 94% reduction</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Insurance BPA may require Lean Six Sigma/BPMN</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Verify Lean/BPMN not day-one</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>pacific life insurance|senior business process analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GR-019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Revenue Operations Analyst / Salesforce Administrator</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Redox</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>$75,000-$95,000</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/redoxengine/d6f780ee-9232-40ab-a478-4cbd0ba7b981</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/redoxengine/d6f780ee-9232-40ab-a478-4cbd0ba7b981</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Revenue Operations/CRM Ops</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>HOLD FOR ARTIFACT</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Proactive data-quality resolution ($4M+ recovery); GTM tool admin (HubSpot); cross-team ops</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>'Administrator' half - verify no Flow/Apex day-one</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Screen SF build requirements</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>redox|revenue operations analyst / salesforce administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GR-020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Digital Marketing Operations Specialist</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Acrisure</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Remote US</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>~$45,500-$59,900 est</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Acrisure Workday</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>https://acrisure.wd1.myworkdayjobs.com/en-US/Acrisure/job/Digital-Marketing-Operations-Specialist_JR113699</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>https://acrisure.wd1.myworkdayjobs.com/en-US/Acrisure/job/Digital-Marketing-Operations-Specialist_JR113699</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Demand Gen/Marketing Operations</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>2</v>
+      </c>
+      <c r="P21" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>HOLD FOR ARTIFACT</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>HubSpot RevOps cert; SOP/workflow automation; cross-functional marketing coordination</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Comp modest for MBA; HubSpot admin depth ramp</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Verify actual comp band</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>acrisure|digital marketing operations specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GR-021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sr Specialist, Marketing Operations - PIM</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Shure</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Remote or Hybrid (Niles IL)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Remote or hybrid</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Verify (hybrid?)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>$87,000-$139,000</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.shure.com/en-US/careers</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.shure.com/en-US/careers</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>MarTech Operations</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>2</v>
+      </c>
+      <c r="P22" t="n">
+        <v>67</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>HOLD FOR ARTIFACT</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>MarTech platform admin + workflow/SOP; analytics/data integrity; AI-assisted workflow</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>PIM/DAM edges toward MDM (not hands-on)</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Possible periodic onsite - verify OH</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>shure|sr specialist, marketing operations - pim</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GR-022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Sales Operations Specialist, Revenue Operations</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>jrni</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Remote US (Boston MA)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>~$95K-$110K est</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ZipRecruiter/jrni</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.jrni.com/careers</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.jrni.com/careers</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Revenue Operations</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P23" t="n">
+        <v>67</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>HOLD FOR ARTIFACT</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Reconcile bookings/billing/revenue ($4M+ recovery); Salesforce data integrity; SOP playbooks</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>CPQ/quote-building + commissions admin net-new</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Sales-facing; confirm not quote-queue</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>jrni|sales operations specialist, revenue operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GR-023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Senior Business Reporting Analyst Lead</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Huntington National Bank</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Columbus OH (remote)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Remote optional US</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Yes (OH employer)</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>$89,300-$115,400</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>https://huntington-jobs.com/</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>https://huntington-jobs.com/</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>2</v>
+      </c>
+      <c r="P24" t="n">
+        <v>66</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Power BI/Tableau + audited reporting; month-end reconciliation; XLOOKUP automation</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>'Lead' may want production SQL/BI ownership</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Verify 'Lead' not people-mgmt</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>huntington national bank|senior business reporting analyst lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GR-024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CRM &amp; Revenue Operations Specialist</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Lee Enterprises / Amplified Digital</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>St. Louis MO</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Full-time direct-hire</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aad6qq96qqtk</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aad6qq96qqtk</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CRM Operations</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>2</v>
+      </c>
+      <c r="P25" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>HOLD FOR ARTIFACT</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Data quality/governance + dedupe/SOP; media/advertising domain; HubSpot workflows/RevOps cert</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Only 2 yrs req (under-levels MBA); email build/deploy</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>~6wk old (may be filled); remote unconfirmed</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>lee enterprises / amplified digital|crm &amp; revenue operations specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GR-025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Business Analyst (Pharma &amp; Life Sciences)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>EVERSANA</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Mason OH (remote or in-office)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Remote or in-office US</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Yes (OH employer)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>$85,000-$115,000</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Built In/ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>https://builtin.com/job/business-analyst/6953058</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>https://builtin.com/job/business-analyst/6953058</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Compliance/Pharma Ops</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>2</v>
+      </c>
+      <c r="P26" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>FDA/PhRMA compliance; QA protocol authorship; cross-functional SOP/reqs</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Agile/Jira BA-ceremony heavy; 5yr BA + 2yr pharma</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Verify open (Built In cache stale)</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>eversana|business analyst (pharma &amp; life sciences)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GR-026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Business Insights Analyst</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Payliance</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Remote US (Columbus OH)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yes (OH employer)</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>$85,000-$115,000</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.payliance.com/careers</t>
+        </is>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.payliance.com/careers</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Reporting Analyst</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>3</v>
+      </c>
+      <c r="P27" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>SELECTIVE STRETCH</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Power BI/Tableau reporting; billing/invoice reconciliation ($4M+); XLOOKUP automation</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Payments SQL may exceed training; domain shift</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Confirm SQL training-acceptable</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>payliance|business insights analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GR-027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Media Analyst I</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Mindgruve</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Remote US (Charleston SC)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Remote optional US</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>$56,500-$73,000</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L28" s="9" t="inlineStr">
+        <is>
+          <t>https://mindgruve.com/careers/</t>
+        </is>
+      </c>
+      <c r="M28" s="9" t="inlineStr">
+        <is>
+          <t>https://mindgruve.com/careers/</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Paid Media/Media Operations</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>2</v>
+      </c>
+      <c r="P28" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DO NOT APPLY</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Omnichannel trafficking/QA/pacing; Power BI/Tableau/GA4; MediaOcean/Prisma/Sizmek</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>AGENCY client-escalation; Analyst I junior/under-leveled</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>High agency reprioritization risk</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>mindgruve|media analyst i</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GR-028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Campaign Operations &amp; Performance Analyst</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Everyday Health Group</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Remote US (NY)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Yes (pending)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>~$60K-$90K est</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Jobvite/JobLeads</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.jobvite.com/everyday-health-consumer</t>
+        </is>
+      </c>
+      <c r="M29" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.jobvite.com/everyday-health-consumer</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Media/Campaign Operations</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>1</v>
+      </c>
+      <c r="P29" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>HOLD FOR ARTIFACT</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Healthcare media campaign ops; Salesforce + GA4; pacing/inventory + coordination</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Targets 1-2 yrs (junior/under-leveled)</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Verify open + remote-in-OH; screen ad-ops tone</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>everyday health group|campaign operations &amp; performance analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GR-029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Senior Finance Analyst, FP&amp;A</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sherwin-Williams</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Cleveland OH (remote)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Remote optional US</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Yes (OH employer)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>$82,900-$103,300</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ZipRecruiter</t>
+        </is>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>https://careers.sherwin-williams.com/</t>
+        </is>
+      </c>
+      <c r="M30" s="9" t="inlineStr">
+        <is>
+          <t>https://careers.sherwin-williams.com/</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Operations/Reporting Analyst (Finance)</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>2</v>
+      </c>
+      <c r="P30" t="n">
+        <v>63</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DO NOT APPLY</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Budget forecasting/financial controls; reconciliation; XLOOKUP + Power BI</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>FP&amp;A GL/accounting-heavy; wants FP&amp;A tenure</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Domain mismatch vs ops-reporting</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>sherwin-williams|senior finance analyst, fp&amp;a</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GR-030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Senior Marketing Operations Manager</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Tiugo Technologies</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Remote US (Boston MA)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>$78,200-$137,400</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Recruitee</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>https://tiugotech.recruitee.com/o/senior-marketing-operations-manager</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>https://tiugotech.recruitee.com/o/senior-marketing-operations-manager</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>MarTech/Marketing Operations</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>3</v>
+      </c>
+      <c r="P31" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DO NOT APPLY</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Lead-lifecycle/campaign process standardization; reporting/attribution; enablement</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Platform build/architecture across 4 brands (over-scoped)</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Martech engineering beyond evidence</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>tiugo technologies|senior marketing operations manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GR-031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Revenue Operations Analyst (RevOps) - Salesforce</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Informativ</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Council Bluffs IA</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Unclear (onsite/hybrid?)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/revenue-operations-analyst-revops-%E2%80%93-salesforce-at-informativ-4432814296</t>
+        </is>
+      </c>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/revenue-operations-analyst-revops-%E2%80%93-salesforce-at-informativ-4432814296</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Revenue Operations/Salesforce Ops</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>2</v>
+      </c>
+      <c r="P32" t="n">
+        <v>62</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>DO NOT APPLY</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>CRM data accuracy; Salesforce reports/dashboards; pipeline velocity</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>5+ yrs rev/sales ops specifically; SaaS pref</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Remote NOT confirmed (IA)</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Provisional pending Phase-3 verification</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>informativ|revenue operations analyst (revops) - salesforce</t>
         </is>
       </c>
     </row>
@@ -1182,6 +4969,70 @@
       <formula1>"Not Started,Prepared - Awaiting Approval,Approved to Submit,Submitted,Interviewing,Rejected,Withdrawn,Expired"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phase 3-5: apply live-verification, archive dead roles, session report
- Verified 15 shortlist postings; 11 live, 3 closed (M3 USA, Viz.ai, Arctic Wolf), 1 unverified (KPA)
- Archived closed roles; downgraded Allstate (social-impact/people-leadership/travel) and KPA
- Added Search Log verification pass + 2026-07-10 session report
- 4 PRIORITY APPLY confirmed live (SureCost, Paylocity, Progressive, 1Password)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EDRVMJpCj9m8Xg2jAMcbUq
</commit_message>
<xml_diff>
--- a/output/Gregory_Reinhart_Job_Search_Tracker.xlsx
+++ b/output/Gregory_Reinhart_Job_Search_Tracker.xlsx
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -957,6 +957,117 @@
       <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GR-009</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>M3 USA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Data Analyst, Pharma/Health/Wellness Media</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Expired + production SQL/Snowflake/Python/dbt screen-out</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>M3 SmartRecruiters</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Verified closed during Phase-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GR-010</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Viz.ai</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Marketing Operations Manager</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>No live MOps role; Pardot/Sr-Mgr</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>viz.ai/jobs</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Verified closed during Phase-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GR-013</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Arctic Wolf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Marketing Performance Analyst</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Posting removed Nov 2025; not live</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Arctic Wolf Workday</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Verified closed during Phase-3</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1269,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Marketing Operations Manager, Campaigns</t>
@@ -1255,12 +1365,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Fully remote US, 5-day work-hours availability; clean MOps/HubSpot fit; +bonus/RSU.</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1280,7 +1387,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Associate Manager, Operations, Governance &amp; AI Enablement</t>
@@ -1340,16 +1446,16 @@
         <v>1</v>
       </c>
       <c r="P3" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>PRIORITY APPLY</t>
+          <t>APPLY WITH TAILORING</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -1364,7 +1470,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Scope creep toward supervision</t>
+          <t>NOT marketing-ops (social-impact ops/gov/AI); possible people-leadership; 10-15% travel</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -1377,12 +1483,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Allstate Foundation/Social Impact; lists Team Leadership + 10-15% travel. AI-governance fit but confirm IC.</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -1402,7 +1505,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Marketing Operations Manager</t>
@@ -1499,12 +1601,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Ohio explicitly in eligible-states; IC reporting to Sr Marketing Mgr; HubSpot-centric.</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1524,7 +1623,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Marketing Process Analyst Senior</t>
@@ -1608,7 +1706,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Occasional HQ travel; Agile-adjacent</t>
+          <t>Occasional office travel; Agile-adjacent digital product cadence</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1621,12 +1719,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. OH HQ (Mayfield); occasional office travel for meetings/training.</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1646,7 +1741,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Senior Revenue Operations Analyst, Campaign Operations</t>
@@ -1664,7 +1758,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Remote-first US</t>
+          <t>Remote-first US (travel expected)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1730,7 +1824,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Minor periodic travel</t>
+          <t>Travel/in-person engagement expected; 'Senior' attribution depth</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1743,12 +1837,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. In-person engagement/travel expected for 'almost all roles'; OH not excluded.</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1768,7 +1859,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Marketing Operations &amp; Project Manager</t>
@@ -1791,7 +1881,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Likely (verify)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1865,12 +1955,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Remote US (must be US-located/authorized); no state exclusion; stack not specified in posting.</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1890,7 +1977,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Sales Operations Analyst 3</t>
@@ -1908,7 +1994,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Fully remote</t>
+          <t>Remote US (flex/hybrid mention-verify)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1938,7 +2024,7 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aavqd9pj492p</t>
+          <t>https://job-boards.greenhouse.io/vipvermontinformationprocessing2/jobs/5170502007</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1987,12 +2073,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. via Greenhouse; benefits mention flex/hybrid + some Colchester VT listings - CONFIRM true remote; builds quote templates (sales-enablement lean).</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -2012,7 +2095,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Marketing Operations Analyst</t>
@@ -2035,7 +2117,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Likely (verify)</t>
+          <t>Yes (fully remote; hybrid only if &lt;30mi Lehi UT)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2109,12 +2191,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Remote US; a separate Calgary Data-Governance role is a DIFFERENT in-office posting - do not confuse.</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -2134,7 +2213,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Data Analyst, Pharma/Health &amp; Wellness Media</t>
@@ -2203,7 +2281,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>APPLY WITH TAILORING</t>
+          <t>DO NOT APPLY (expired + production SQL/Snowflake/Python/dbt)</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -2228,15 +2306,12 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+          <t>Expired</t>
+        </is>
+      </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>CLOSED 2026-07-10: posting expired AND requires production SQL/Snowflake/Python/dbt (data-science ownership) - screen-out.</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -2256,7 +2331,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Marketing Operations Manager</t>
@@ -2325,7 +2399,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>APPLY WITH TAILORING</t>
+          <t>DO NOT APPLY (no live MOps role)</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -2350,15 +2424,12 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
+          <t>Expired</t>
+        </is>
+      </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>CLOSED 2026-07-10: no Marketing Operations role live on viz.ai/jobs; prior postings Pardot-centric + Senior-Manager (people-mgmt).</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -2378,7 +2449,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Revenue Operations Analyst (CRM &amp; Data Systems)</t>
@@ -2401,7 +2471,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Remote US (OH not named)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2475,12 +2545,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. HubSpot/Dynamics RevOps + data integrity + Clay; cover letter OPTIONAL; no SF-admin/SQL/quota screen-outs.</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -2500,7 +2567,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Revenue Operations Analyst</t>
@@ -2597,12 +2663,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Remote US, no state exclusion; entry-level RevOps: Salesforce+reporting+marketing ops; no Apex/CPQ.</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2622,7 +2685,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Marketing Performance Analyst</t>
@@ -2691,7 +2753,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>SELECTIVE STRETCH</t>
+          <t>DO NOT APPLY (posting removed Nov 2025)</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -2716,15 +2778,12 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
+          <t>Expired</t>
+        </is>
+      </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>CLOSED: removed 2025-11-14; not present in current Arctic Wolf Workday. Reconsider only if it reopens.</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -2744,7 +2803,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>GTM Operations Manager</t>
@@ -2841,12 +2899,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>VERIFIED LIVE 2026-07-10. Fully remote; hands-on Salesforce+HubSpot admin (no Apex/CPQ); SQL preferred not required; 5+ yrs GTM/RevOps, no direct reports/quota.</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2866,7 +2921,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Revenue Operations Analyst</t>
@@ -2935,7 +2989,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>SELECTIVE STRETCH</t>
+          <t>HOLD (unverified live posting)</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2963,12 +3017,9 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Provisional pending Phase-3 verification</t>
+          <t>UNVERIFIED 2026-07-10: could not confirm a live RevOps Analyst posting (JS-rendered careers page; no board listing found); KPA remote-first with occasional required in-office events.</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2988,7 +3039,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>Marketing Specialist (HubSpot Specialization)</t>
@@ -3085,9 +3135,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3110,7 +3157,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>GTM Operations Analyst (Marketing)</t>
@@ -3207,9 +3253,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3232,7 +3275,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Senior Business Process Analyst</t>
@@ -3329,9 +3371,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3354,7 +3393,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Revenue Operations Analyst / Salesforce Administrator</t>
@@ -3451,9 +3489,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
       <c r="AA20" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3476,7 +3511,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Digital Marketing Operations Specialist</t>
@@ -3573,9 +3607,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3598,7 +3629,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>Sr Specialist, Marketing Operations - PIM</t>
@@ -3695,9 +3725,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3720,7 +3747,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Sales Operations Specialist, Revenue Operations</t>
@@ -3817,9 +3843,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3842,7 +3865,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Senior Business Reporting Analyst Lead</t>
@@ -3939,9 +3961,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -3964,7 +3983,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>CRM &amp; Revenue Operations Specialist</t>
@@ -4061,9 +4079,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4086,7 +4101,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Business Analyst (Pharma &amp; Life Sciences)</t>
@@ -4183,9 +4197,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4208,7 +4219,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Business Insights Analyst</t>
@@ -4305,9 +4315,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4330,7 +4337,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Media Analyst I</t>
@@ -4427,9 +4433,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4452,7 +4455,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Campaign Operations &amp; Performance Analyst</t>
@@ -4549,9 +4551,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4574,7 +4573,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Senior Finance Analyst, FP&amp;A</t>
@@ -4671,9 +4669,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4696,7 +4691,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Senior Marketing Operations Manager</t>
@@ -4793,9 +4787,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -4818,7 +4809,6 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Revenue Operations Analyst (RevOps) - Salesforce</t>
@@ -4915,9 +4905,6 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="inlineStr">
         <is>
           <t>Provisional pending Phase-3 verification</t>
@@ -5043,7 +5030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5367,6 +5354,58 @@
       <c r="J6" t="inlineStr">
         <is>
           <t>Dice engineering-heavy; low signal for MarOps — deprioritized</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Employer/ATS pages</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Phase-3 verification of 15 shortlist postings</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>(all shortlist families)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>live-check</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>11 live</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>3 closed (M3,Viz.ai,Arctic Wolf); 1 unverified (KPA)</t>
         </is>
       </c>
     </row>

</xml_diff>